<commit_message>
Full restore uploaded known-good Market Survey 12
</commit_message>
<xml_diff>
--- a/templates/template_by_dealer.xlsx
+++ b/templates/template_by_dealer.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\kb_market_survey\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Bot\KB_Market_Survey_Telegram_V33_14_KHMER_SUMMARY_RENDER_FIXED\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC9F2BA-F99E-47C0-BC0D-C1EEA9F689DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B38315-5AC2-47DC-BA7C-612F87B54A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="94">
   <si>
     <t>Market Improvement Report</t>
   </si>
@@ -248,9 +248,6 @@
   </si>
   <si>
     <t>4.</t>
-  </si>
-  <si>
-    <t>CBC LITE ORD</t>
   </si>
   <si>
     <t>CBC 4.4 NCP</t>
@@ -449,42 +446,42 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -788,134 +785,134 @@
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="12"/>
-      <c r="H2" s="12"/>
-      <c r="I2" s="12"/>
-      <c r="J2" s="12"/>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
-      <c r="N2" s="12"/>
-      <c r="O2" s="12"/>
-      <c r="P2" s="12"/>
-      <c r="Q2" s="12"/>
-      <c r="R2" s="12"/>
-      <c r="S2" s="12"/>
-      <c r="T2" s="12"/>
-      <c r="U2" s="12"/>
-      <c r="V2" s="12"/>
-      <c r="W2" s="12"/>
-      <c r="X2" s="12"/>
-      <c r="Y2" s="12"/>
-      <c r="Z2" s="12"/>
-      <c r="AA2" s="12"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
+      <c r="U2" s="9"/>
+      <c r="V2" s="9"/>
+      <c r="W2" s="9"/>
+      <c r="X2" s="9"/>
+      <c r="Y2" s="9"/>
+      <c r="Z2" s="9"/>
+      <c r="AA2" s="9"/>
     </row>
     <row r="3" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
-      <c r="K3" s="12"/>
-      <c r="L3" s="12"/>
-      <c r="M3" s="12"/>
-      <c r="N3" s="12"/>
-      <c r="O3" s="12"/>
-      <c r="P3" s="12"/>
-      <c r="Q3" s="12"/>
-      <c r="R3" s="12"/>
-      <c r="S3" s="12"/>
-      <c r="T3" s="12"/>
-      <c r="U3" s="12"/>
-      <c r="V3" s="12"/>
-      <c r="W3" s="12"/>
-      <c r="X3" s="12"/>
-      <c r="Y3" s="12"/>
-      <c r="Z3" s="12"/>
-      <c r="AA3" s="12"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+      <c r="U3" s="9"/>
+      <c r="V3" s="9"/>
+      <c r="W3" s="9"/>
+      <c r="X3" s="9"/>
+      <c r="Y3" s="9"/>
+      <c r="Z3" s="9"/>
+      <c r="AA3" s="9"/>
     </row>
     <row r="4" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="8" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="8" t="s">
+      <c r="D4" s="11"/>
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
-      <c r="Q4" s="9"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="9"/>
-      <c r="T4" s="9"/>
-      <c r="U4" s="9"/>
-      <c r="V4" s="10"/>
-      <c r="W4" s="8" t="s">
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+      <c r="N4" s="11"/>
+      <c r="O4" s="11"/>
+      <c r="P4" s="11"/>
+      <c r="Q4" s="11"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="11"/>
+      <c r="T4" s="11"/>
+      <c r="U4" s="11"/>
+      <c r="V4" s="12"/>
+      <c r="W4" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="X4" s="9"/>
-      <c r="Y4" s="9"/>
-      <c r="Z4" s="9"/>
-      <c r="AA4" s="10"/>
+      <c r="X4" s="11"/>
+      <c r="Y4" s="11"/>
+      <c r="Z4" s="11"/>
+      <c r="AA4" s="12"/>
     </row>
     <row r="5" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
-      <c r="I5" s="9"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="9"/>
-      <c r="O5" s="9"/>
-      <c r="P5" s="9"/>
-      <c r="Q5" s="9"/>
-      <c r="R5" s="9"/>
-      <c r="S5" s="9"/>
-      <c r="T5" s="9"/>
-      <c r="U5" s="9"/>
-      <c r="V5" s="9"/>
-      <c r="W5" s="9"/>
-      <c r="X5" s="9"/>
-      <c r="Y5" s="9"/>
-      <c r="Z5" s="9"/>
-      <c r="AA5" s="10"/>
+      <c r="B5" s="11"/>
+      <c r="C5" s="11"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+      <c r="N5" s="11"/>
+      <c r="O5" s="11"/>
+      <c r="P5" s="11"/>
+      <c r="Q5" s="11"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="11"/>
+      <c r="T5" s="11"/>
+      <c r="U5" s="11"/>
+      <c r="V5" s="11"/>
+      <c r="W5" s="11"/>
+      <c r="X5" s="11"/>
+      <c r="Y5" s="11"/>
+      <c r="Z5" s="11"/>
+      <c r="AA5" s="12"/>
     </row>
     <row r="6" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="2" t="s">
@@ -924,210 +921,210 @@
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="14" t="s">
+      <c r="D6" s="11"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="14" t="s">
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="12"/>
+      <c r="L6" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="10"/>
-      <c r="P6" s="14" t="s">
+      <c r="M6" s="11"/>
+      <c r="N6" s="11"/>
+      <c r="O6" s="12"/>
+      <c r="P6" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="Q6" s="9"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="10"/>
-      <c r="T6" s="14" t="s">
+      <c r="Q6" s="11"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="12"/>
+      <c r="T6" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="U6" s="9"/>
-      <c r="V6" s="10"/>
-      <c r="W6" s="20" t="s">
+      <c r="U6" s="11"/>
+      <c r="V6" s="12"/>
+      <c r="W6" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="X6" s="9"/>
-      <c r="Y6" s="10"/>
-      <c r="Z6" s="20" t="s">
+      <c r="X6" s="11"/>
+      <c r="Y6" s="12"/>
+      <c r="Z6" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="AA6" s="10"/>
+      <c r="AA6" s="12"/>
     </row>
     <row r="7" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="3">
         <v>1</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="10"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="9"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="10"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="9"/>
-      <c r="V7" s="10"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="9"/>
-      <c r="Y7" s="10"/>
-      <c r="Z7" s="13"/>
-      <c r="AA7" s="10"/>
+        <v>84</v>
+      </c>
+      <c r="C7" s="10"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="11"/>
+      <c r="N7" s="11"/>
+      <c r="O7" s="12"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="11"/>
+      <c r="R7" s="11"/>
+      <c r="S7" s="12"/>
+      <c r="T7" s="10"/>
+      <c r="U7" s="11"/>
+      <c r="V7" s="12"/>
+      <c r="W7" s="10"/>
+      <c r="X7" s="11"/>
+      <c r="Y7" s="12"/>
+      <c r="Z7" s="10"/>
+      <c r="AA7" s="12"/>
     </row>
     <row r="8" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="3">
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C8" s="13"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="13"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="13"/>
-      <c r="M8" s="9"/>
-      <c r="N8" s="9"/>
-      <c r="O8" s="10"/>
-      <c r="P8" s="13"/>
-      <c r="Q8" s="9"/>
-      <c r="R8" s="9"/>
-      <c r="S8" s="10"/>
-      <c r="T8" s="13"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="10"/>
-      <c r="W8" s="13"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="10"/>
-      <c r="Z8" s="13"/>
-      <c r="AA8" s="10"/>
+        <v>76</v>
+      </c>
+      <c r="C8" s="10"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="11"/>
+      <c r="N8" s="11"/>
+      <c r="O8" s="12"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="11"/>
+      <c r="R8" s="11"/>
+      <c r="S8" s="12"/>
+      <c r="T8" s="10"/>
+      <c r="U8" s="11"/>
+      <c r="V8" s="12"/>
+      <c r="W8" s="10"/>
+      <c r="X8" s="11"/>
+      <c r="Y8" s="12"/>
+      <c r="Z8" s="10"/>
+      <c r="AA8" s="12"/>
     </row>
     <row r="9" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="3">
         <v>3</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="10"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="9"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="10"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="10"/>
-      <c r="W9" s="13"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="10"/>
-      <c r="Z9" s="13"/>
-      <c r="AA9" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="C9" s="10"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="12"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="11"/>
+      <c r="R9" s="11"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="10"/>
+      <c r="U9" s="11"/>
+      <c r="V9" s="12"/>
+      <c r="W9" s="10"/>
+      <c r="X9" s="11"/>
+      <c r="Y9" s="12"/>
+      <c r="Z9" s="10"/>
+      <c r="AA9" s="12"/>
     </row>
     <row r="10" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="3">
         <v>4</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="13"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="13"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="13"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="10"/>
-      <c r="P10" s="13"/>
-      <c r="Q10" s="9"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="13"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="10"/>
-      <c r="W10" s="13"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="10"/>
-      <c r="Z10" s="13"/>
-      <c r="AA10" s="10"/>
+        <v>78</v>
+      </c>
+      <c r="C10" s="10"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="11"/>
+      <c r="R10" s="11"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="10"/>
+      <c r="U10" s="11"/>
+      <c r="V10" s="12"/>
+      <c r="W10" s="10"/>
+      <c r="X10" s="11"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="10"/>
+      <c r="AA10" s="12"/>
     </row>
     <row r="11" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>5</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="9"/>
-      <c r="N11" s="9"/>
-      <c r="O11" s="10"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="9"/>
-      <c r="R11" s="9"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="13"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="10"/>
-      <c r="W11" s="13"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="10"/>
-      <c r="Z11" s="13"/>
-      <c r="AA11" s="10"/>
+        <v>79</v>
+      </c>
+      <c r="C11" s="10"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="10"/>
+      <c r="Q11" s="11"/>
+      <c r="R11" s="11"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="10"/>
+      <c r="U11" s="11"/>
+      <c r="V11" s="12"/>
+      <c r="W11" s="10"/>
+      <c r="X11" s="11"/>
+      <c r="Y11" s="12"/>
+      <c r="Z11" s="10"/>
+      <c r="AA11" s="12"/>
     </row>
     <row r="12" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
@@ -1136,31 +1133,31 @@
       <c r="B12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="13"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="13"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="10"/>
-      <c r="P12" s="13"/>
-      <c r="Q12" s="9"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="10"/>
-      <c r="T12" s="13"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="10"/>
-      <c r="W12" s="13"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="10"/>
-      <c r="Z12" s="13"/>
-      <c r="AA12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="10"/>
+      <c r="Q12" s="11"/>
+      <c r="R12" s="11"/>
+      <c r="S12" s="12"/>
+      <c r="T12" s="10"/>
+      <c r="U12" s="11"/>
+      <c r="V12" s="12"/>
+      <c r="W12" s="10"/>
+      <c r="X12" s="11"/>
+      <c r="Y12" s="12"/>
+      <c r="Z12" s="10"/>
+      <c r="AA12" s="12"/>
     </row>
     <row r="13" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
@@ -1169,64 +1166,64 @@
       <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="13"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="13"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="10"/>
-      <c r="P13" s="13"/>
-      <c r="Q13" s="9"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="10"/>
-      <c r="T13" s="13"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="10"/>
-      <c r="W13" s="13"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="10"/>
-      <c r="Z13" s="13"/>
-      <c r="AA13" s="10"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="10"/>
+      <c r="Q13" s="11"/>
+      <c r="R13" s="11"/>
+      <c r="S13" s="12"/>
+      <c r="T13" s="10"/>
+      <c r="U13" s="11"/>
+      <c r="V13" s="12"/>
+      <c r="W13" s="10"/>
+      <c r="X13" s="11"/>
+      <c r="Y13" s="12"/>
+      <c r="Z13" s="10"/>
+      <c r="AA13" s="12"/>
     </row>
     <row r="14" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>8</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="13"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="10"/>
-      <c r="P14" s="13"/>
-      <c r="Q14" s="9"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="10"/>
-      <c r="T14" s="13"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="10"/>
-      <c r="W14" s="13"/>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="10"/>
-      <c r="Z14" s="13"/>
-      <c r="AA14" s="10"/>
+        <v>80</v>
+      </c>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="10"/>
+      <c r="Q14" s="11"/>
+      <c r="R14" s="11"/>
+      <c r="S14" s="12"/>
+      <c r="T14" s="10"/>
+      <c r="U14" s="11"/>
+      <c r="V14" s="12"/>
+      <c r="W14" s="10"/>
+      <c r="X14" s="11"/>
+      <c r="Y14" s="12"/>
+      <c r="Z14" s="10"/>
+      <c r="AA14" s="12"/>
     </row>
     <row r="15" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
@@ -1235,31 +1232,31 @@
       <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="13"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="13"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="13"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="10"/>
-      <c r="P15" s="13"/>
-      <c r="Q15" s="9"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="10"/>
-      <c r="T15" s="13"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="10"/>
-      <c r="W15" s="13"/>
-      <c r="X15" s="9"/>
-      <c r="Y15" s="10"/>
-      <c r="Z15" s="13"/>
-      <c r="AA15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="10"/>
+      <c r="Q15" s="11"/>
+      <c r="R15" s="11"/>
+      <c r="S15" s="12"/>
+      <c r="T15" s="10"/>
+      <c r="U15" s="11"/>
+      <c r="V15" s="12"/>
+      <c r="W15" s="10"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="12"/>
+      <c r="Z15" s="10"/>
+      <c r="AA15" s="12"/>
     </row>
     <row r="16" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
@@ -1268,31 +1265,31 @@
       <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C16" s="13"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="13"/>
-      <c r="Q16" s="9"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="10"/>
-      <c r="T16" s="13"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="10"/>
-      <c r="W16" s="13"/>
-      <c r="X16" s="9"/>
-      <c r="Y16" s="10"/>
-      <c r="Z16" s="13"/>
-      <c r="AA16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="12"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="11"/>
+      <c r="O16" s="12"/>
+      <c r="P16" s="10"/>
+      <c r="Q16" s="11"/>
+      <c r="R16" s="11"/>
+      <c r="S16" s="12"/>
+      <c r="T16" s="10"/>
+      <c r="U16" s="11"/>
+      <c r="V16" s="12"/>
+      <c r="W16" s="10"/>
+      <c r="X16" s="11"/>
+      <c r="Y16" s="12"/>
+      <c r="Z16" s="10"/>
+      <c r="AA16" s="12"/>
     </row>
     <row r="17" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
@@ -1301,31 +1298,31 @@
       <c r="B17" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="13"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="13"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="10"/>
-      <c r="P17" s="13"/>
-      <c r="Q17" s="9"/>
-      <c r="R17" s="9"/>
-      <c r="S17" s="10"/>
-      <c r="T17" s="13"/>
-      <c r="U17" s="9"/>
-      <c r="V17" s="10"/>
-      <c r="W17" s="13"/>
-      <c r="X17" s="9"/>
-      <c r="Y17" s="10"/>
-      <c r="Z17" s="13"/>
-      <c r="AA17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="12"/>
+      <c r="L17" s="10"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="11"/>
+      <c r="O17" s="12"/>
+      <c r="P17" s="10"/>
+      <c r="Q17" s="11"/>
+      <c r="R17" s="11"/>
+      <c r="S17" s="12"/>
+      <c r="T17" s="10"/>
+      <c r="U17" s="11"/>
+      <c r="V17" s="12"/>
+      <c r="W17" s="10"/>
+      <c r="X17" s="11"/>
+      <c r="Y17" s="12"/>
+      <c r="Z17" s="10"/>
+      <c r="AA17" s="12"/>
     </row>
     <row r="18" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
@@ -1334,64 +1331,64 @@
       <c r="B18" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="10"/>
-      <c r="P18" s="13"/>
-      <c r="Q18" s="9"/>
-      <c r="R18" s="9"/>
-      <c r="S18" s="10"/>
-      <c r="T18" s="13"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="10"/>
-      <c r="W18" s="13"/>
-      <c r="X18" s="9"/>
-      <c r="Y18" s="10"/>
-      <c r="Z18" s="13"/>
-      <c r="AA18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="12"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="11"/>
+      <c r="O18" s="12"/>
+      <c r="P18" s="10"/>
+      <c r="Q18" s="11"/>
+      <c r="R18" s="11"/>
+      <c r="S18" s="12"/>
+      <c r="T18" s="10"/>
+      <c r="U18" s="11"/>
+      <c r="V18" s="12"/>
+      <c r="W18" s="10"/>
+      <c r="X18" s="11"/>
+      <c r="Y18" s="12"/>
+      <c r="Z18" s="10"/>
+      <c r="AA18" s="12"/>
     </row>
     <row r="19" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>13</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="10"/>
-      <c r="P19" s="13"/>
-      <c r="Q19" s="9"/>
-      <c r="R19" s="9"/>
-      <c r="S19" s="10"/>
-      <c r="T19" s="13"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="10"/>
-      <c r="W19" s="13"/>
-      <c r="X19" s="9"/>
-      <c r="Y19" s="10"/>
-      <c r="Z19" s="13"/>
-      <c r="AA19" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="C19" s="10"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="12"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="11"/>
+      <c r="O19" s="12"/>
+      <c r="P19" s="10"/>
+      <c r="Q19" s="11"/>
+      <c r="R19" s="11"/>
+      <c r="S19" s="12"/>
+      <c r="T19" s="10"/>
+      <c r="U19" s="11"/>
+      <c r="V19" s="12"/>
+      <c r="W19" s="10"/>
+      <c r="X19" s="11"/>
+      <c r="Y19" s="12"/>
+      <c r="Z19" s="10"/>
+      <c r="AA19" s="12"/>
     </row>
     <row r="20" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
@@ -1400,31 +1397,31 @@
       <c r="B20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="13"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="13"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="10"/>
-      <c r="P20" s="13"/>
-      <c r="Q20" s="9"/>
-      <c r="R20" s="9"/>
-      <c r="S20" s="10"/>
-      <c r="T20" s="13"/>
-      <c r="U20" s="9"/>
-      <c r="V20" s="10"/>
-      <c r="W20" s="13"/>
-      <c r="X20" s="9"/>
-      <c r="Y20" s="10"/>
-      <c r="Z20" s="13"/>
-      <c r="AA20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="11"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="10"/>
+      <c r="Q20" s="11"/>
+      <c r="R20" s="11"/>
+      <c r="S20" s="12"/>
+      <c r="T20" s="10"/>
+      <c r="U20" s="11"/>
+      <c r="V20" s="12"/>
+      <c r="W20" s="10"/>
+      <c r="X20" s="11"/>
+      <c r="Y20" s="12"/>
+      <c r="Z20" s="10"/>
+      <c r="AA20" s="12"/>
     </row>
     <row r="21" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
@@ -1433,31 +1430,31 @@
       <c r="B21" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="13"/>
-      <c r="D21" s="9"/>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="10"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="9"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="10"/>
-      <c r="P21" s="13"/>
-      <c r="Q21" s="9"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="10"/>
-      <c r="T21" s="13"/>
-      <c r="U21" s="9"/>
-      <c r="V21" s="10"/>
-      <c r="W21" s="13"/>
-      <c r="X21" s="9"/>
-      <c r="Y21" s="10"/>
-      <c r="Z21" s="13"/>
-      <c r="AA21" s="10"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="10"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="11"/>
+      <c r="O21" s="12"/>
+      <c r="P21" s="10"/>
+      <c r="Q21" s="11"/>
+      <c r="R21" s="11"/>
+      <c r="S21" s="12"/>
+      <c r="T21" s="10"/>
+      <c r="U21" s="11"/>
+      <c r="V21" s="12"/>
+      <c r="W21" s="10"/>
+      <c r="X21" s="11"/>
+      <c r="Y21" s="12"/>
+      <c r="Z21" s="10"/>
+      <c r="AA21" s="12"/>
     </row>
     <row r="22" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
@@ -1466,31 +1463,31 @@
       <c r="B22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="13"/>
-      <c r="D22" s="9"/>
-      <c r="E22" s="9"/>
-      <c r="F22" s="9"/>
-      <c r="G22" s="10"/>
-      <c r="H22" s="13"/>
-      <c r="I22" s="9"/>
-      <c r="J22" s="9"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="13"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="10"/>
-      <c r="P22" s="13"/>
-      <c r="Q22" s="9"/>
-      <c r="R22" s="9"/>
-      <c r="S22" s="10"/>
-      <c r="T22" s="13"/>
-      <c r="U22" s="9"/>
-      <c r="V22" s="10"/>
-      <c r="W22" s="13"/>
-      <c r="X22" s="9"/>
-      <c r="Y22" s="10"/>
-      <c r="Z22" s="13"/>
-      <c r="AA22" s="10"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="11"/>
+      <c r="O22" s="12"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="11"/>
+      <c r="R22" s="11"/>
+      <c r="S22" s="12"/>
+      <c r="T22" s="10"/>
+      <c r="U22" s="11"/>
+      <c r="V22" s="12"/>
+      <c r="W22" s="10"/>
+      <c r="X22" s="11"/>
+      <c r="Y22" s="12"/>
+      <c r="Z22" s="10"/>
+      <c r="AA22" s="12"/>
     </row>
     <row r="23" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
@@ -1499,31 +1496,31 @@
       <c r="B23" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="10"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="9"/>
-      <c r="N23" s="9"/>
-      <c r="O23" s="10"/>
-      <c r="P23" s="13"/>
-      <c r="Q23" s="9"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="10"/>
-      <c r="T23" s="13"/>
-      <c r="U23" s="9"/>
-      <c r="V23" s="10"/>
-      <c r="W23" s="13"/>
-      <c r="X23" s="9"/>
-      <c r="Y23" s="10"/>
-      <c r="Z23" s="13"/>
-      <c r="AA23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="10"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="11"/>
+      <c r="O23" s="12"/>
+      <c r="P23" s="10"/>
+      <c r="Q23" s="11"/>
+      <c r="R23" s="11"/>
+      <c r="S23" s="12"/>
+      <c r="T23" s="10"/>
+      <c r="U23" s="11"/>
+      <c r="V23" s="12"/>
+      <c r="W23" s="10"/>
+      <c r="X23" s="11"/>
+      <c r="Y23" s="12"/>
+      <c r="Z23" s="10"/>
+      <c r="AA23" s="12"/>
     </row>
     <row r="24" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
@@ -1532,62 +1529,62 @@
       <c r="B24" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="13"/>
-      <c r="D24" s="9"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="10"/>
-      <c r="H24" s="13"/>
-      <c r="I24" s="9"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="9"/>
-      <c r="N24" s="9"/>
-      <c r="O24" s="10"/>
-      <c r="P24" s="13"/>
-      <c r="Q24" s="9"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="10"/>
-      <c r="T24" s="13"/>
-      <c r="U24" s="9"/>
-      <c r="V24" s="10"/>
-      <c r="W24" s="13"/>
-      <c r="X24" s="9"/>
-      <c r="Y24" s="10"/>
-      <c r="Z24" s="13"/>
-      <c r="AA24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="10"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="11"/>
+      <c r="O24" s="12"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="11"/>
+      <c r="R24" s="11"/>
+      <c r="S24" s="12"/>
+      <c r="T24" s="10"/>
+      <c r="U24" s="11"/>
+      <c r="V24" s="12"/>
+      <c r="W24" s="10"/>
+      <c r="X24" s="11"/>
+      <c r="Y24" s="12"/>
+      <c r="Z24" s="10"/>
+      <c r="AA24" s="12"/>
     </row>
     <row r="25" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="12"/>
-      <c r="K25" s="12"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="12"/>
-      <c r="N25" s="12"/>
-      <c r="O25" s="12"/>
-      <c r="P25" s="12"/>
-      <c r="Q25" s="12"/>
-      <c r="R25" s="12"/>
-      <c r="S25" s="12"/>
-      <c r="T25" s="12"/>
-      <c r="U25" s="12"/>
-      <c r="V25" s="12"/>
-      <c r="W25" s="12"/>
-      <c r="X25" s="12"/>
-      <c r="Y25" s="12"/>
-      <c r="Z25" s="12"/>
-      <c r="AA25" s="12"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="9"/>
+      <c r="T25" s="9"/>
+      <c r="U25" s="9"/>
+      <c r="V25" s="9"/>
+      <c r="W25" s="9"/>
+      <c r="X25" s="9"/>
+      <c r="Y25" s="9"/>
+      <c r="Z25" s="9"/>
+      <c r="AA25" s="9"/>
     </row>
     <row r="26" spans="1:27" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="4" t="s">
@@ -1677,7 +1674,7 @@
         <v>1</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1685,21 +1682,21 @@
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
       <c r="H27" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I27" s="3"/>
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="N27" s="3"/>
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
       <c r="R27" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="S27" s="3"/>
       <c r="T27" s="3"/>
@@ -1716,7 +1713,7 @@
         <v>2</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1724,21 +1721,21 @@
       <c r="F28" s="3"/>
       <c r="G28" s="3"/>
       <c r="H28" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I28" s="3"/>
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N28" s="3"/>
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
       <c r="R28" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="S28" s="3"/>
       <c r="T28" s="3"/>
@@ -1755,7 +1752,7 @@
         <v>3</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1763,28 +1760,28 @@
       <c r="F29" s="3"/>
       <c r="G29" s="3"/>
       <c r="H29" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I29" s="3"/>
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N29" s="3"/>
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
       <c r="R29" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="S29" s="3"/>
       <c r="T29" s="3"/>
       <c r="U29" s="3"/>
       <c r="V29" s="3"/>
       <c r="W29" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="X29" s="3"/>
       <c r="Y29" s="3"/>
@@ -1796,7 +1793,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1809,7 +1806,7 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N30" s="3"/>
       <c r="O30" s="3"/>
@@ -1918,7 +1915,7 @@
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="N33" s="3"/>
       <c r="O33" s="3"/>
@@ -1942,7 +1939,7 @@
         <v>8</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -2127,7 +2124,7 @@
         <v>13</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -2283,187 +2280,330 @@
       <c r="AA42" s="3"/>
     </row>
     <row r="43" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B43" s="12"/>
-      <c r="C43" s="12"/>
-      <c r="D43" s="12"/>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" spans="1:27" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B44" s="19" t="s">
+      <c r="B44" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C44" s="10"/>
-      <c r="D44" s="21" t="s">
+      <c r="C44" s="12"/>
+      <c r="D44" s="16" t="s">
         <v>67</v>
       </c>
-      <c r="E44" s="10"/>
-      <c r="F44" s="18" t="s">
+      <c r="E44" s="12"/>
+      <c r="F44" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="G44" s="10"/>
-      <c r="I44" s="11" t="s">
+      <c r="G44" s="12"/>
+      <c r="I44" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="J44" s="12"/>
-      <c r="K44" s="12"/>
-      <c r="L44" s="12"/>
-      <c r="M44" s="12"/>
-      <c r="N44" s="12"/>
-      <c r="O44" s="12"/>
-      <c r="P44" s="12"/>
-      <c r="Q44" s="12"/>
-      <c r="S44" s="11" t="s">
+      <c r="J44" s="9"/>
+      <c r="K44" s="9"/>
+      <c r="L44" s="9"/>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
+      <c r="P44" s="9"/>
+      <c r="Q44" s="9"/>
+      <c r="S44" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="T44" s="12"/>
-      <c r="U44" s="12"/>
-      <c r="V44" s="12"/>
-      <c r="W44" s="12"/>
-      <c r="X44" s="12"/>
-      <c r="Y44" s="12"/>
-      <c r="Z44" s="12"/>
-      <c r="AA44" s="12"/>
+      <c r="T44" s="9"/>
+      <c r="U44" s="9"/>
+      <c r="V44" s="9"/>
+      <c r="W44" s="9"/>
+      <c r="X44" s="9"/>
+      <c r="Y44" s="9"/>
+      <c r="Z44" s="9"/>
+      <c r="AA44" s="9"/>
     </row>
     <row r="45" spans="1:27" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="3">
         <v>1</v>
       </c>
-      <c r="B45" s="22" t="s">
+      <c r="B45" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C45" s="10"/>
-      <c r="D45" s="13"/>
-      <c r="E45" s="10"/>
-      <c r="F45" s="13"/>
-      <c r="G45" s="10"/>
-      <c r="I45" s="16">
+      <c r="C45" s="12"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="12"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="12"/>
+      <c r="I45" s="13">
         <v>1</v>
       </c>
-      <c r="J45" s="12"/>
-      <c r="K45" s="12"/>
-      <c r="L45" s="12"/>
-      <c r="M45" s="12"/>
-      <c r="N45" s="12"/>
-      <c r="O45" s="12"/>
-      <c r="P45" s="12"/>
-      <c r="Q45" s="12"/>
-      <c r="S45" s="16">
+      <c r="J45" s="9"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="9"/>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9"/>
+      <c r="O45" s="9"/>
+      <c r="P45" s="9"/>
+      <c r="Q45" s="9"/>
+      <c r="S45" s="13">
         <v>1</v>
       </c>
-      <c r="T45" s="12"/>
-      <c r="U45" s="12"/>
-      <c r="V45" s="12"/>
-      <c r="W45" s="12"/>
-      <c r="X45" s="12"/>
-      <c r="Y45" s="12"/>
-      <c r="Z45" s="12"/>
-      <c r="AA45" s="12"/>
+      <c r="T45" s="9"/>
+      <c r="U45" s="9"/>
+      <c r="V45" s="9"/>
+      <c r="W45" s="9"/>
+      <c r="X45" s="9"/>
+      <c r="Y45" s="9"/>
+      <c r="Z45" s="9"/>
+      <c r="AA45" s="9"/>
     </row>
     <row r="46" spans="1:27" ht="62.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="3">
         <v>2</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C46" s="10"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="13"/>
-      <c r="G46" s="10"/>
-      <c r="I46" s="16" t="s">
+      <c r="C46" s="12"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="12"/>
+      <c r="F46" s="10"/>
+      <c r="G46" s="12"/>
+      <c r="I46" s="13" t="s">
         <v>73</v>
       </c>
-      <c r="J46" s="12"/>
-      <c r="K46" s="12"/>
-      <c r="L46" s="12"/>
-      <c r="M46" s="12"/>
-      <c r="N46" s="12"/>
-      <c r="O46" s="12"/>
-      <c r="P46" s="12"/>
-      <c r="Q46" s="12"/>
-      <c r="S46" s="16">
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="9"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
+      <c r="O46" s="9"/>
+      <c r="P46" s="9"/>
+      <c r="Q46" s="9"/>
+      <c r="S46" s="13">
         <v>2</v>
       </c>
-      <c r="T46" s="12"/>
-      <c r="U46" s="12"/>
-      <c r="V46" s="12"/>
-      <c r="W46" s="12"/>
-      <c r="X46" s="12"/>
-      <c r="Y46" s="12"/>
-      <c r="Z46" s="12"/>
-      <c r="AA46" s="12"/>
+      <c r="T46" s="9"/>
+      <c r="U46" s="9"/>
+      <c r="V46" s="9"/>
+      <c r="W46" s="9"/>
+      <c r="X46" s="9"/>
+      <c r="Y46" s="9"/>
+      <c r="Z46" s="9"/>
+      <c r="AA46" s="9"/>
     </row>
     <row r="47" spans="1:27" ht="72.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="5"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="12"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="12"/>
-      <c r="F47" s="17"/>
-      <c r="G47" s="12"/>
-      <c r="I47" s="16" t="s">
+      <c r="B47" s="8"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="9"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="9"/>
+      <c r="I47" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="J47" s="12"/>
-      <c r="K47" s="12"/>
-      <c r="L47" s="12"/>
-      <c r="M47" s="12"/>
-      <c r="N47" s="12"/>
-      <c r="O47" s="12"/>
-      <c r="P47" s="12"/>
-      <c r="Q47" s="12"/>
-      <c r="S47" s="16">
+      <c r="J47" s="9"/>
+      <c r="K47" s="9"/>
+      <c r="L47" s="9"/>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+      <c r="O47" s="9"/>
+      <c r="P47" s="9"/>
+      <c r="Q47" s="9"/>
+      <c r="S47" s="13">
         <v>3</v>
       </c>
-      <c r="T47" s="12"/>
-      <c r="U47" s="12"/>
-      <c r="V47" s="12"/>
-      <c r="W47" s="12"/>
-      <c r="X47" s="12"/>
-      <c r="Y47" s="12"/>
-      <c r="Z47" s="12"/>
-      <c r="AA47" s="12"/>
+      <c r="T47" s="9"/>
+      <c r="U47" s="9"/>
+      <c r="V47" s="9"/>
+      <c r="W47" s="9"/>
+      <c r="X47" s="9"/>
+      <c r="Y47" s="9"/>
+      <c r="Z47" s="9"/>
+      <c r="AA47" s="9"/>
     </row>
     <row r="48" spans="1:27" ht="95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="5"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="12"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="12"/>
-      <c r="F48" s="17"/>
-      <c r="G48" s="12"/>
-      <c r="I48" s="16" t="s">
+      <c r="B48" s="8"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="9"/>
+      <c r="I48" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="J48" s="12"/>
-      <c r="K48" s="12"/>
-      <c r="L48" s="12"/>
-      <c r="M48" s="12"/>
-      <c r="N48" s="12"/>
-      <c r="O48" s="12"/>
-      <c r="P48" s="12"/>
-      <c r="Q48" s="12"/>
-      <c r="S48" s="16" t="s">
+      <c r="J48" s="9"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="9"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="9"/>
+      <c r="O48" s="9"/>
+      <c r="P48" s="9"/>
+      <c r="Q48" s="9"/>
+      <c r="S48" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="T48" s="12"/>
-      <c r="U48" s="12"/>
-      <c r="V48" s="12"/>
-      <c r="W48" s="12"/>
-      <c r="X48" s="12"/>
-      <c r="Y48" s="12"/>
-      <c r="Z48" s="12"/>
-      <c r="AA48" s="12"/>
+      <c r="T48" s="9"/>
+      <c r="U48" s="9"/>
+      <c r="V48" s="9"/>
+      <c r="W48" s="9"/>
+      <c r="X48" s="9"/>
+      <c r="Y48" s="9"/>
+      <c r="Z48" s="9"/>
+      <c r="AA48" s="9"/>
     </row>
     <row r="49" ht="25" customHeight="1" x14ac:dyDescent="0.35"/>
   </sheetData>
   <mergeCells count="167">
+    <mergeCell ref="I44:Q44"/>
+    <mergeCell ref="L18:O18"/>
+    <mergeCell ref="P11:S11"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="Z13:AA13"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="T20:V20"/>
+    <mergeCell ref="P10:S10"/>
+    <mergeCell ref="W4:AA4"/>
+    <mergeCell ref="L6:O6"/>
+    <mergeCell ref="Z8:AA8"/>
+    <mergeCell ref="L8:O8"/>
+    <mergeCell ref="T8:V8"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="Z19:AA19"/>
+    <mergeCell ref="Z9:AA9"/>
+    <mergeCell ref="W15:Y15"/>
+    <mergeCell ref="Z18:AA18"/>
+    <mergeCell ref="W24:Y24"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="T19:V19"/>
+    <mergeCell ref="W14:Y14"/>
+    <mergeCell ref="L19:O19"/>
+    <mergeCell ref="A2:AA2"/>
+    <mergeCell ref="T23:V23"/>
+    <mergeCell ref="W19:Y19"/>
+    <mergeCell ref="P21:S21"/>
+    <mergeCell ref="I46:Q46"/>
+    <mergeCell ref="W9:Y9"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="L20:O20"/>
+    <mergeCell ref="Z22:AA22"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="P23:S23"/>
+    <mergeCell ref="L13:O13"/>
+    <mergeCell ref="Z24:AA24"/>
+    <mergeCell ref="A43:D43"/>
+    <mergeCell ref="P6:S6"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="Z14:AA14"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="T21:V21"/>
+    <mergeCell ref="C8:G8"/>
+    <mergeCell ref="L15:O15"/>
+    <mergeCell ref="T15:V15"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="I48:Q48"/>
+    <mergeCell ref="S48:AA48"/>
+    <mergeCell ref="Z16:AA16"/>
+    <mergeCell ref="H4:V4"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="W21:Y21"/>
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="L22:O22"/>
+    <mergeCell ref="W23:Y23"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="I45:Q45"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="H19:K19"/>
+    <mergeCell ref="W13:Y13"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="W22:Y22"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="T9:V9"/>
+    <mergeCell ref="W10:Y10"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="T18:V18"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="L17:O17"/>
+    <mergeCell ref="Z23:AA23"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="Z15:AA15"/>
+    <mergeCell ref="P12:S12"/>
+    <mergeCell ref="W11:Y11"/>
+    <mergeCell ref="H18:K18"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="I47:Q47"/>
+    <mergeCell ref="S44:AA44"/>
+    <mergeCell ref="L21:O21"/>
+    <mergeCell ref="H20:K20"/>
+    <mergeCell ref="L23:O23"/>
+    <mergeCell ref="P14:S14"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="T13:V13"/>
+    <mergeCell ref="T22:V22"/>
+    <mergeCell ref="P16:S16"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="Z17:AA17"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="T24:V24"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="T14:V14"/>
+    <mergeCell ref="T17:V17"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="L9:O9"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="Z21:AA21"/>
+    <mergeCell ref="Z6:AA6"/>
+    <mergeCell ref="C6:G6"/>
+    <mergeCell ref="L10:O10"/>
+    <mergeCell ref="T10:V10"/>
+    <mergeCell ref="P8:S8"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="Z10:AA10"/>
+    <mergeCell ref="P19:S19"/>
+    <mergeCell ref="Z12:AA12"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="W8:Y8"/>
+    <mergeCell ref="W17:Y17"/>
+    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="L7:O7"/>
+    <mergeCell ref="P7:S7"/>
+    <mergeCell ref="T7:V7"/>
+    <mergeCell ref="W7:Y7"/>
+    <mergeCell ref="Z7:AA7"/>
+    <mergeCell ref="C4:G4"/>
+    <mergeCell ref="S45:AA45"/>
+    <mergeCell ref="W16:Y16"/>
+    <mergeCell ref="P18:S18"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="H17:K17"/>
+    <mergeCell ref="L11:O11"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="P20:S20"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="L24:O24"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="P24:S24"/>
+    <mergeCell ref="Z11:AA11"/>
+    <mergeCell ref="A25:AA25"/>
+    <mergeCell ref="Z20:AA20"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="P17:S17"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="T11:V11"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="B45:C45"/>
+    <mergeCell ref="B46:C46"/>
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="P13:S13"/>
     <mergeCell ref="D48:E48"/>
@@ -2488,149 +2628,6 @@
     <mergeCell ref="L16:O16"/>
     <mergeCell ref="T16:V16"/>
     <mergeCell ref="C18:G18"/>
-    <mergeCell ref="S45:AA45"/>
-    <mergeCell ref="W16:Y16"/>
-    <mergeCell ref="P18:S18"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="H17:K17"/>
-    <mergeCell ref="L11:O11"/>
-    <mergeCell ref="C14:G14"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="P20:S20"/>
-    <mergeCell ref="C16:G16"/>
-    <mergeCell ref="L24:O24"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="P24:S24"/>
-    <mergeCell ref="Z11:AA11"/>
-    <mergeCell ref="A25:AA25"/>
-    <mergeCell ref="Z20:AA20"/>
-    <mergeCell ref="C20:G20"/>
-    <mergeCell ref="P17:S17"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="T11:V11"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="B45:C45"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="L9:O9"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Z21:AA21"/>
-    <mergeCell ref="Z6:AA6"/>
-    <mergeCell ref="C6:G6"/>
-    <mergeCell ref="L10:O10"/>
-    <mergeCell ref="T10:V10"/>
-    <mergeCell ref="P8:S8"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="Z10:AA10"/>
-    <mergeCell ref="P19:S19"/>
-    <mergeCell ref="Z12:AA12"/>
-    <mergeCell ref="C15:G15"/>
-    <mergeCell ref="W8:Y8"/>
-    <mergeCell ref="W17:Y17"/>
-    <mergeCell ref="C7:G7"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="L7:O7"/>
-    <mergeCell ref="P7:S7"/>
-    <mergeCell ref="T7:V7"/>
-    <mergeCell ref="W7:Y7"/>
-    <mergeCell ref="Z7:AA7"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="Z15:AA15"/>
-    <mergeCell ref="P12:S12"/>
-    <mergeCell ref="W11:Y11"/>
-    <mergeCell ref="H18:K18"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="I47:Q47"/>
-    <mergeCell ref="S44:AA44"/>
-    <mergeCell ref="L21:O21"/>
-    <mergeCell ref="H20:K20"/>
-    <mergeCell ref="L23:O23"/>
-    <mergeCell ref="P14:S14"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="T13:V13"/>
-    <mergeCell ref="T22:V22"/>
-    <mergeCell ref="P16:S16"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="Z17:AA17"/>
-    <mergeCell ref="C11:G11"/>
-    <mergeCell ref="C17:G17"/>
-    <mergeCell ref="T24:V24"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="T14:V14"/>
-    <mergeCell ref="T17:V17"/>
-    <mergeCell ref="I48:Q48"/>
-    <mergeCell ref="S48:AA48"/>
-    <mergeCell ref="Z16:AA16"/>
-    <mergeCell ref="H4:V4"/>
-    <mergeCell ref="C19:G19"/>
-    <mergeCell ref="W21:Y21"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="L22:O22"/>
-    <mergeCell ref="W23:Y23"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="I45:Q45"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="H19:K19"/>
-    <mergeCell ref="W13:Y13"/>
-    <mergeCell ref="C21:G21"/>
-    <mergeCell ref="W22:Y22"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="T9:V9"/>
-    <mergeCell ref="W10:Y10"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="T18:V18"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="L17:O17"/>
-    <mergeCell ref="Z23:AA23"/>
-    <mergeCell ref="A2:AA2"/>
-    <mergeCell ref="T23:V23"/>
-    <mergeCell ref="W19:Y19"/>
-    <mergeCell ref="P21:S21"/>
-    <mergeCell ref="I46:Q46"/>
-    <mergeCell ref="W9:Y9"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="L20:O20"/>
-    <mergeCell ref="Z22:AA22"/>
-    <mergeCell ref="C22:G22"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="P23:S23"/>
-    <mergeCell ref="L13:O13"/>
-    <mergeCell ref="Z24:AA24"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="P6:S6"/>
-    <mergeCell ref="C24:G24"/>
-    <mergeCell ref="Z14:AA14"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="T21:V21"/>
-    <mergeCell ref="C8:G8"/>
-    <mergeCell ref="L15:O15"/>
-    <mergeCell ref="T15:V15"/>
-    <mergeCell ref="C23:G23"/>
-    <mergeCell ref="C4:G4"/>
-    <mergeCell ref="I44:Q44"/>
-    <mergeCell ref="L18:O18"/>
-    <mergeCell ref="P11:S11"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="Z13:AA13"/>
-    <mergeCell ref="C13:G13"/>
-    <mergeCell ref="T20:V20"/>
-    <mergeCell ref="P10:S10"/>
-    <mergeCell ref="W4:AA4"/>
-    <mergeCell ref="L6:O6"/>
-    <mergeCell ref="Z8:AA8"/>
-    <mergeCell ref="L8:O8"/>
-    <mergeCell ref="T8:V8"/>
-    <mergeCell ref="C10:G10"/>
-    <mergeCell ref="Z19:AA19"/>
-    <mergeCell ref="Z9:AA9"/>
-    <mergeCell ref="W15:Y15"/>
-    <mergeCell ref="Z18:AA18"/>
-    <mergeCell ref="W24:Y24"/>
-    <mergeCell ref="C12:G12"/>
-    <mergeCell ref="T19:V19"/>
-    <mergeCell ref="W14:Y14"/>
-    <mergeCell ref="L19:O19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>